<commit_message>
end of day, progess made
</commit_message>
<xml_diff>
--- a/team_wins_vs_salary.xlsx
+++ b/team_wins_vs_salary.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BolognaColonel\workspace\SQL\group-projects\newforce-cohort-12-data-lahmanbaseball-The-Greenbrier-Batboys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F9D7BA04-956D-4B8F-AA9C-F290D7D96ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4C83A337-AB76-4A30-A3EB-A39FB9D37ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="600" windowWidth="28800" windowHeight="21000" xr2:uid="{00DFF9BB-299D-4DD7-B595-A38CD862CFF2}"/>
+    <workbookView xWindow="4800" yWindow="0" windowWidth="28800" windowHeight="21000" xr2:uid="{00DFF9BB-299D-4DD7-B595-A38CD862CFF2}"/>
   </bookViews>
   <sheets>
     <sheet name="team_wins_salaries" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="team_wins_attendance" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="37">
   <si>
     <t>teamid</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>MON</t>
+  </si>
+  <si>
+    <t>total_attend</t>
   </si>
 </sst>
 </file>
@@ -780,7 +783,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>team_wins_salaries!$B$39</c:f>
+              <c:f>team_wins_salaries!$B$38</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -803,7 +806,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>team_wins_salaries!$A$40:$A$72</c:f>
+              <c:f>team_wins_salaries!$A$39:$A$71</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
@@ -910,7 +913,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>team_wins_salaries!$B$40:$B$72</c:f>
+              <c:f>team_wins_salaries!$B$39:$B$71</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
@@ -1044,7 +1047,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>team_wins_salaries!$C$39</c:f>
+              <c:f>team_wins_salaries!$C$38</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1067,7 +1070,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>team_wins_salaries!$A$40:$A$72</c:f>
+              <c:f>team_wins_salaries!$A$39:$A$71</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
@@ -1174,7 +1177,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>team_wins_salaries!$C$40:$C$72</c:f>
+              <c:f>team_wins_salaries!$C$39:$C$71</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="33"/>
@@ -2405,6 +2408,1716 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Team</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Total Wins (DESC) Vs. Total Attendance</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>team_wins_attendance!$B$38</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>total_wins</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>team_wins_attendance!$A$39:$A$71</c:f>
+              <c:strCache>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>NYA</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>SLN</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>BOS</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>LAN</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>ATL</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OAK</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>SFN</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>PHI</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>TEX</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>CHA</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>TOR</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>MIN</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>CLE</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>CHN</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>NYN</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>SEA</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>DET</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>ARI</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>HOU</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>CIN</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>SDN</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>MIL</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>TBA</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>BAL</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>COL</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>PIT</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>KCA</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>LAA</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>WAS</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>FLO</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>MIA</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>ANA</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>MON</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>team_wins_attendance!$B$39:$B$71</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>1505</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1455</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1422</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1393</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1381</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1369</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1365</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1345</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1325</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1304</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1295</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1295</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1288</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1281</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1269</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1257</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1253</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1238</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1231</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1225</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1221</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1219</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1203</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1190</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1178</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1156</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1065</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>950</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>884</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>358</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>343</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>301</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-ED97-4243-9A02-A01F0AEF0FC8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="873181456"/>
+        <c:axId val="873182896"/>
+      </c:lineChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>team_wins_attendance!$C$38</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>total_attend</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>team_wins_attendance!$A$39:$A$71</c:f>
+              <c:strCache>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>NYA</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>SLN</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>BOS</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>LAN</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>ATL</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>OAK</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>SFN</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>PHI</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>TEX</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>CHA</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>TOR</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>MIN</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>CLE</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>CHN</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>NYN</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>SEA</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>DET</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>ARI</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>HOU</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>CIN</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>SDN</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>MIL</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>TBA</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>BAL</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>COL</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>PIT</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>KCA</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>LAA</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>WAS</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>FLO</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>MIA</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>ANA</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>MON</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>team_wins_attendance!$C$39:$C$71</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>58495152</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>52888435</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46466930</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>56302147</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>39101975</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>29479543</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>51584001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44495437</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41172841</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>33164590</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>34849294</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>36979419</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>30397034</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>47961695</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44014864</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>39654117</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>39498837</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>37031107</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>38980402</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>34266878</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>37887696</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>40930678</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22728889</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>36688181</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>41290884</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>31148454</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>28092982</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>38377383</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>27455620</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>15333536</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>9002701</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>10740557</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3229469</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-ED97-4243-9A02-A01F0AEF0FC8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1748150991"/>
+        <c:axId val="904905872"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="873181456"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="873182896"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="873182896"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="873181456"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="904905872"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1748150991"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="1748150991"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="904905872"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Team Total Attendance (DESC) Vs. Total Wins</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>team_wins_attendance!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>total_attend</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>team_wins_attendance!$A$2:$A$34</c:f>
+              <c:strCache>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>NYA</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>LAN</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>SLN</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>SFN</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>CHN</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>BOS</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>PHI</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>NYN</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>COL</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>TEX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>MIL</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>SEA</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>DET</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>ATL</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>HOU</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>LAA</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>SDN</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>ARI</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>MIN</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>BAL</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>TOR</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>CIN</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>CHA</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>PIT</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>CLE</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>OAK</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>KCA</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>WAS</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>TBA</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>FLO</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>ANA</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>MIA</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>MON</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>team_wins_attendance!$C$2:$C$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>58495152</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>56302147</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>52888435</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>51584001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>47961695</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46466930</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44495437</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44014864</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41290884</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>41172841</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>40930678</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>39654117</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>39498837</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>39101975</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>38980402</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>38377383</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>37887696</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>37031107</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>36979419</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>36688181</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>34849294</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>34266878</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>33164590</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>31148454</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>30397034</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>29479543</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>28092982</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27455620</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22728889</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>15333536</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10740557</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>9002701</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3229469</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A701-4CBD-B4F1-4F1F6BB92F15}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="857092944"/>
+        <c:axId val="857090544"/>
+      </c:lineChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>team_wins_attendance!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>total_wins</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>team_wins_attendance!$A$2:$A$34</c:f>
+              <c:strCache>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>NYA</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>LAN</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>SLN</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>SFN</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>CHN</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>BOS</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>PHI</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>NYN</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>COL</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>TEX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>MIL</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>SEA</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>DET</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>ATL</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>HOU</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>LAA</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>SDN</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>ARI</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>MIN</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>BAL</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>TOR</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>CIN</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>CHA</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>PIT</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>CLE</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>OAK</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>KCA</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>WAS</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>TBA</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>FLO</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>ANA</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>MIA</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>MON</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>team_wins_attendance!$B$2:$B$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="33"/>
+                <c:pt idx="0">
+                  <c:v>1505</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1393</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1455</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1365</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1288</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1422</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1345</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1281</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1190</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1325</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1221</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1269</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1257</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1381</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1238</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1065</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1225</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1253</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1295</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1203</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1231</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1304</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1178</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1295</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1369</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1156</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>950</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1219</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>884</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>343</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>358</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>301</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A701-4CBD-B4F1-4F1F6BB92F15}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1076986975"/>
+        <c:axId val="1076986015"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="857092944"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="857090544"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="857090544"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="857092944"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1076986015"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1076986975"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="1076986975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1076986015"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2485,6 +4198,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
@@ -3517,19 +5310,1025 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>454025</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>71</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3574,6 +6373,83 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF3773C6-2490-74C1-56E4-2F4D3F78933C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>14286</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>417513</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57844166-5512-EAA8-D3D4-18874B90495D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>4761</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>409574</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>181926</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FAD257A5-6472-67D1-C320-0D55C1F30BA0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3911,7 +6787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71912485-71A6-4A3B-BDD1-0F1F5E6C720F}">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="22" customWidth="1"/>
@@ -3930,7 +6806,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:C34">_xlfn._xlws.SORT(A40:C72, 3,-1)</f>
+        <f t="array" ref="A2:C34">_xlfn._xlws.SORT(A39:C71, 3,-1)</f>
         <v>NYA</v>
       </c>
       <c r="B2">
@@ -4292,377 +7168,377 @@
         <v>166676000</v>
       </c>
     </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2</v>
+      </c>
+    </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="B39">
+        <v>1505</v>
+      </c>
+      <c r="C39" s="1">
+        <v>3047137657</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B40">
-        <v>1505</v>
+        <v>1455</v>
       </c>
       <c r="C40" s="1">
-        <v>3047137657</v>
+        <v>1564175387</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B41">
-        <v>1455</v>
+        <v>1422</v>
       </c>
       <c r="C41" s="1">
-        <v>1564175387</v>
+        <v>2244609605</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B42">
-        <v>1422</v>
+        <v>1393</v>
       </c>
       <c r="C42" s="1">
-        <v>2244609605</v>
+        <v>2083523132</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B43">
-        <v>1393</v>
+        <v>1381</v>
       </c>
       <c r="C43" s="1">
-        <v>2083523132</v>
+        <v>1424245926</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44">
-        <v>1381</v>
+        <v>1369</v>
       </c>
       <c r="C44" s="1">
-        <v>1424245926</v>
+        <v>965978860</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B45">
-        <v>1369</v>
+        <v>1365</v>
       </c>
       <c r="C45" s="1">
-        <v>965978860</v>
+        <v>1711653388</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B46">
-        <v>1365</v>
+        <v>1345</v>
       </c>
       <c r="C46" s="1">
-        <v>1711653388</v>
+        <v>1758350323</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B47">
-        <v>1345</v>
+        <v>1325</v>
       </c>
       <c r="C47" s="1">
-        <v>1758350323</v>
+        <v>1493609120</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B48">
-        <v>1325</v>
+        <v>1304</v>
       </c>
       <c r="C48" s="1">
-        <v>1493609120</v>
+        <v>1500293976</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B49">
-        <v>1304</v>
+        <v>1300</v>
       </c>
       <c r="C49" s="1">
-        <v>1500293976</v>
+        <v>1320119132</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B50">
-        <v>1300</v>
+        <v>1295</v>
       </c>
       <c r="C50" s="1">
-        <v>1320119132</v>
+        <v>1160717904</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51">
         <v>1295</v>
       </c>
       <c r="C51" s="1">
-        <v>1160717904</v>
+        <v>1083032280</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B52">
-        <v>1295</v>
+        <v>1288</v>
       </c>
       <c r="C52" s="1">
-        <v>1083032280</v>
+        <v>1641008162</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B53">
-        <v>1288</v>
+        <v>1281</v>
       </c>
       <c r="C53" s="1">
-        <v>1641008162</v>
+        <v>1718420612</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B54">
-        <v>1281</v>
+        <v>1269</v>
       </c>
       <c r="C54" s="1">
-        <v>1718420612</v>
+        <v>1501251033</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B55">
-        <v>1269</v>
+        <v>1257</v>
       </c>
       <c r="C55" s="1">
-        <v>1501251033</v>
+        <v>1730611133</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B56">
-        <v>1257</v>
+        <v>1253</v>
       </c>
       <c r="C56" s="1">
-        <v>1730611133</v>
+        <v>1177169459</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B57">
-        <v>1253</v>
+        <v>1238</v>
       </c>
       <c r="C57" s="1">
-        <v>1177169459</v>
+        <v>1159514747</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B58">
-        <v>1238</v>
+        <v>1231</v>
       </c>
       <c r="C58" s="1">
-        <v>1159514747</v>
+        <v>1185557183</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B59">
-        <v>1231</v>
+        <v>1225</v>
       </c>
       <c r="C59" s="1">
-        <v>1185557183</v>
+        <v>989561977</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B60">
-        <v>1225</v>
+        <v>1221</v>
       </c>
       <c r="C60" s="1">
-        <v>989561977</v>
+        <v>1103988658</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B61">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="C61" s="1">
-        <v>1103988658</v>
+        <v>760814289</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B62">
-        <v>1219</v>
+        <v>1203</v>
       </c>
       <c r="C62" s="1">
-        <v>760814289</v>
+        <v>1336554654</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B63">
-        <v>1203</v>
+        <v>1190</v>
       </c>
       <c r="C63" s="1">
-        <v>1336554654</v>
+        <v>1176577595</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B64">
-        <v>1190</v>
+        <v>1178</v>
       </c>
       <c r="C64" s="1">
-        <v>1176577595</v>
+        <v>897749487</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B65">
-        <v>1178</v>
+        <v>1156</v>
       </c>
       <c r="C65" s="1">
-        <v>897749487</v>
+        <v>1017176218</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B66">
-        <v>1156</v>
+        <v>1065</v>
       </c>
       <c r="C66" s="1">
-        <v>1017176218</v>
+        <v>1441928434</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B67">
-        <v>1065</v>
+        <v>950</v>
       </c>
       <c r="C67" s="1">
-        <v>1441928434</v>
+        <v>1012600139</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B68">
-        <v>950</v>
+        <v>884</v>
       </c>
       <c r="C68" s="1">
-        <v>1012600139</v>
+        <v>447542012</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B69">
-        <v>884</v>
+        <v>358</v>
       </c>
       <c r="C69" s="1">
-        <v>447542012</v>
+        <v>338887502</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B70">
-        <v>358</v>
+        <v>343</v>
       </c>
       <c r="C70" s="1">
-        <v>338887502</v>
+        <v>288823168</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B71">
-        <v>343</v>
+        <v>301</v>
       </c>
       <c r="C71" s="1">
-        <v>288823168</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>35</v>
-      </c>
-      <c r="B72">
-        <v>301</v>
-      </c>
-      <c r="C72" s="1">
         <v>166676000</v>
       </c>
     </row>
@@ -4673,11 +7549,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12DF9993-7E9E-4656-8D6E-9C01217705B5}">
-  <dimension ref="A1:C34"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17950D09-160E-418A-AF5D-1B639D7EDC25}">
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -4688,373 +7564,749 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
+      <c r="A2" t="str" cm="1">
+        <f t="array" ref="A2:C34">_xlfn._xlws.SORT(A39:C71, 3,-1)</f>
+        <v>NYA</v>
       </c>
       <c r="B2">
         <v>1505</v>
       </c>
-      <c r="C2" s="1">
-        <v>3047137657</v>
+      <c r="C2">
+        <v>58495152</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
+      <c r="A3" t="str">
+        <v>LAN</v>
       </c>
       <c r="B3">
+        <v>1393</v>
+      </c>
+      <c r="C3">
+        <v>56302147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <v>SLN</v>
+      </c>
+      <c r="B4">
         <v>1455</v>
       </c>
-      <c r="C3" s="1">
-        <v>1564175387</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
+      <c r="C4">
+        <v>52888435</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <v>SFN</v>
+      </c>
+      <c r="B5">
+        <v>1365</v>
+      </c>
+      <c r="C5">
+        <v>51584001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <v>CHN</v>
+      </c>
+      <c r="B6">
+        <v>1288</v>
+      </c>
+      <c r="C6">
+        <v>47961695</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <v>BOS</v>
+      </c>
+      <c r="B7">
         <v>1422</v>
       </c>
-      <c r="C4" s="1">
-        <v>2244609605</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>1393</v>
-      </c>
-      <c r="C5" s="1">
-        <v>2083523132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
+      <c r="C7">
+        <v>46466930</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <v>PHI</v>
+      </c>
+      <c r="B8">
+        <v>1345</v>
+      </c>
+      <c r="C8">
+        <v>44495437</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <v>NYN</v>
+      </c>
+      <c r="B9">
+        <v>1281</v>
+      </c>
+      <c r="C9">
+        <v>44014864</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <v>COL</v>
+      </c>
+      <c r="B10">
+        <v>1190</v>
+      </c>
+      <c r="C10">
+        <v>41290884</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <v>TEX</v>
+      </c>
+      <c r="B11">
+        <v>1325</v>
+      </c>
+      <c r="C11">
+        <v>41172841</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <v>MIL</v>
+      </c>
+      <c r="B12">
+        <v>1221</v>
+      </c>
+      <c r="C12">
+        <v>40930678</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <v>SEA</v>
+      </c>
+      <c r="B13">
+        <v>1269</v>
+      </c>
+      <c r="C13">
+        <v>39654117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <v>DET</v>
+      </c>
+      <c r="B14">
+        <v>1257</v>
+      </c>
+      <c r="C14">
+        <v>39498837</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <v>ATL</v>
+      </c>
+      <c r="B15">
         <v>1381</v>
       </c>
-      <c r="C6" s="1">
-        <v>1424245926</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>1369</v>
-      </c>
-      <c r="C7" s="1">
-        <v>965978860</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>1365</v>
-      </c>
-      <c r="C8" s="1">
-        <v>1711653388</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>1345</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1758350323</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10">
-        <v>1325</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1493609120</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11">
-        <v>1304</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1500293976</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12">
-        <v>1300</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1320119132</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13">
-        <v>1295</v>
-      </c>
-      <c r="C13" s="1">
-        <v>1160717904</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14">
-        <v>1295</v>
-      </c>
-      <c r="C14" s="1">
-        <v>1083032280</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15">
-        <v>1288</v>
-      </c>
-      <c r="C15" s="1">
-        <v>1641008162</v>
+      <c r="C15">
+        <v>39101975</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>17</v>
+      <c r="A16" t="str">
+        <v>HOU</v>
       </c>
       <c r="B16">
-        <v>1281</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1718420612</v>
+        <v>1238</v>
+      </c>
+      <c r="C16">
+        <v>38980402</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>18</v>
+      <c r="A17" t="str">
+        <v>LAA</v>
       </c>
       <c r="B17">
-        <v>1269</v>
-      </c>
-      <c r="C17" s="1">
-        <v>1501251033</v>
+        <v>1065</v>
+      </c>
+      <c r="C17">
+        <v>38377383</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>19</v>
+      <c r="A18" t="str">
+        <v>SDN</v>
       </c>
       <c r="B18">
-        <v>1257</v>
-      </c>
-      <c r="C18" s="1">
-        <v>1730611133</v>
+        <v>1225</v>
+      </c>
+      <c r="C18">
+        <v>37887696</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>20</v>
+      <c r="A19" t="str">
+        <v>ARI</v>
       </c>
       <c r="B19">
         <v>1253</v>
       </c>
-      <c r="C19" s="1">
-        <v>1177169459</v>
+      <c r="C19">
+        <v>37031107</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>21</v>
+      <c r="A20" t="str">
+        <v>MIN</v>
       </c>
       <c r="B20">
-        <v>1238</v>
-      </c>
-      <c r="C20" s="1">
-        <v>1159514747</v>
+        <v>1295</v>
+      </c>
+      <c r="C20">
+        <v>36979419</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>22</v>
+      <c r="A21" t="str">
+        <v>BAL</v>
       </c>
       <c r="B21">
+        <v>1203</v>
+      </c>
+      <c r="C21">
+        <v>36688181</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <v>TOR</v>
+      </c>
+      <c r="B22">
+        <v>1300</v>
+      </c>
+      <c r="C22">
+        <v>34849294</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <v>CIN</v>
+      </c>
+      <c r="B23">
         <v>1231</v>
       </c>
-      <c r="C21" s="1">
-        <v>1185557183</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22">
-        <v>1225</v>
-      </c>
-      <c r="C22" s="1">
-        <v>989561977</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23">
-        <v>1221</v>
-      </c>
-      <c r="C23" s="1">
-        <v>1103988658</v>
+      <c r="C23">
+        <v>34266878</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>25</v>
+      <c r="A24" t="str">
+        <v>CHA</v>
       </c>
       <c r="B24">
-        <v>1219</v>
-      </c>
-      <c r="C24" s="1">
-        <v>760814289</v>
+        <v>1304</v>
+      </c>
+      <c r="C24">
+        <v>33164590</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>26</v>
+      <c r="A25" t="str">
+        <v>PIT</v>
       </c>
       <c r="B25">
-        <v>1203</v>
-      </c>
-      <c r="C25" s="1">
-        <v>1336554654</v>
+        <v>1178</v>
+      </c>
+      <c r="C25">
+        <v>31148454</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>27</v>
+      <c r="A26" t="str">
+        <v>CLE</v>
       </c>
       <c r="B26">
-        <v>1190</v>
-      </c>
-      <c r="C26" s="1">
-        <v>1176577595</v>
+        <v>1295</v>
+      </c>
+      <c r="C26">
+        <v>30397034</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>28</v>
+      <c r="A27" t="str">
+        <v>OAK</v>
       </c>
       <c r="B27">
-        <v>1178</v>
-      </c>
-      <c r="C27" s="1">
-        <v>897749487</v>
+        <v>1369</v>
+      </c>
+      <c r="C27">
+        <v>29479543</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>29</v>
+      <c r="A28" t="str">
+        <v>KCA</v>
       </c>
       <c r="B28">
         <v>1156</v>
       </c>
-      <c r="C28" s="1">
-        <v>1017176218</v>
+      <c r="C28">
+        <v>28092982</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>30</v>
+      <c r="A29" t="str">
+        <v>WAS</v>
       </c>
       <c r="B29">
-        <v>1065</v>
-      </c>
-      <c r="C29" s="1">
-        <v>1441928434</v>
+        <v>950</v>
+      </c>
+      <c r="C29">
+        <v>27455620</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>31</v>
+      <c r="A30" t="str">
+        <v>TBA</v>
       </c>
       <c r="B30">
-        <v>950</v>
-      </c>
-      <c r="C30" s="1">
-        <v>1012600139</v>
+        <v>1219</v>
+      </c>
+      <c r="C30">
+        <v>22728889</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>32</v>
+      <c r="A31" t="str">
+        <v>FLO</v>
       </c>
       <c r="B31">
         <v>884</v>
       </c>
-      <c r="C31" s="1">
-        <v>447542012</v>
+      <c r="C31">
+        <v>15333536</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>33</v>
+      <c r="A32" t="str">
+        <v>ANA</v>
       </c>
       <c r="B32">
+        <v>343</v>
+      </c>
+      <c r="C32">
+        <v>10740557</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="str">
+        <v>MIA</v>
+      </c>
+      <c r="B33">
         <v>358</v>
       </c>
-      <c r="C32" s="1">
-        <v>338887502</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33">
-        <v>343</v>
-      </c>
-      <c r="C33" s="1">
-        <v>288823168</v>
+      <c r="C33">
+        <v>9002701</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>35</v>
+      <c r="A34" t="str">
+        <v>MON</v>
       </c>
       <c r="B34">
         <v>301</v>
       </c>
-      <c r="C34" s="1">
-        <v>166676000</v>
+      <c r="C34">
+        <v>3229469</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39">
+        <v>1505</v>
+      </c>
+      <c r="C39">
+        <v>58495152</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40">
+        <v>1455</v>
+      </c>
+      <c r="C40">
+        <v>52888435</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41">
+        <v>1422</v>
+      </c>
+      <c r="C41">
+        <v>46466930</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42">
+        <v>1393</v>
+      </c>
+      <c r="C42">
+        <v>56302147</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43">
+        <v>1381</v>
+      </c>
+      <c r="C43">
+        <v>39101975</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>8</v>
+      </c>
+      <c r="B44">
+        <v>1369</v>
+      </c>
+      <c r="C44">
+        <v>29479543</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45">
+        <v>1365</v>
+      </c>
+      <c r="C45">
+        <v>51584001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>10</v>
+      </c>
+      <c r="B46">
+        <v>1345</v>
+      </c>
+      <c r="C46">
+        <v>44495437</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47">
+        <v>1325</v>
+      </c>
+      <c r="C47">
+        <v>41172841</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48">
+        <v>1304</v>
+      </c>
+      <c r="C48">
+        <v>33164590</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49">
+        <v>1300</v>
+      </c>
+      <c r="C49">
+        <v>34849294</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B50">
+        <v>1295</v>
+      </c>
+      <c r="C50">
+        <v>36979419</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51">
+        <v>1295</v>
+      </c>
+      <c r="C51">
+        <v>30397034</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52">
+        <v>1288</v>
+      </c>
+      <c r="C52">
+        <v>47961695</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53">
+        <v>1281</v>
+      </c>
+      <c r="C53">
+        <v>44014864</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54">
+        <v>1269</v>
+      </c>
+      <c r="C54">
+        <v>39654117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55">
+        <v>1257</v>
+      </c>
+      <c r="C55">
+        <v>39498837</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56">
+        <v>1253</v>
+      </c>
+      <c r="C56">
+        <v>37031107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>21</v>
+      </c>
+      <c r="B57">
+        <v>1238</v>
+      </c>
+      <c r="C57">
+        <v>38980402</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>22</v>
+      </c>
+      <c r="B58">
+        <v>1231</v>
+      </c>
+      <c r="C58">
+        <v>34266878</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>23</v>
+      </c>
+      <c r="B59">
+        <v>1225</v>
+      </c>
+      <c r="C59">
+        <v>37887696</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>24</v>
+      </c>
+      <c r="B60">
+        <v>1221</v>
+      </c>
+      <c r="C60">
+        <v>40930678</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>25</v>
+      </c>
+      <c r="B61">
+        <v>1219</v>
+      </c>
+      <c r="C61">
+        <v>22728889</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>26</v>
+      </c>
+      <c r="B62">
+        <v>1203</v>
+      </c>
+      <c r="C62">
+        <v>36688181</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>27</v>
+      </c>
+      <c r="B63">
+        <v>1190</v>
+      </c>
+      <c r="C63">
+        <v>41290884</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>28</v>
+      </c>
+      <c r="B64">
+        <v>1178</v>
+      </c>
+      <c r="C64">
+        <v>31148454</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>29</v>
+      </c>
+      <c r="B65">
+        <v>1156</v>
+      </c>
+      <c r="C65">
+        <v>28092982</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>30</v>
+      </c>
+      <c r="B66">
+        <v>1065</v>
+      </c>
+      <c r="C66">
+        <v>38377383</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>31</v>
+      </c>
+      <c r="B67">
+        <v>950</v>
+      </c>
+      <c r="C67">
+        <v>27455620</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>32</v>
+      </c>
+      <c r="B68">
+        <v>884</v>
+      </c>
+      <c r="C68">
+        <v>15333536</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>33</v>
+      </c>
+      <c r="B69">
+        <v>358</v>
+      </c>
+      <c r="C69">
+        <v>9002701</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>34</v>
+      </c>
+      <c r="B70">
+        <v>343</v>
+      </c>
+      <c r="C70">
+        <v>10740557</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>35</v>
+      </c>
+      <c r="B71">
+        <v>301</v>
+      </c>
+      <c r="C71">
+        <v>3229469</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>